<commit_message>
v2: text dimensions, pieces, pallet/overhang notes, top-load fairness fix, de-narrated policy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168G8qEcectCjGAHz28F1s9
</commit_message>
<xml_diff>
--- a/bus-b44-b2-ltl-freight-class-quote-selection/solution/files/quote_selection.xlsx
+++ b/bus-b44-b2-ltl-freight-class-quote-selection/solution/files/quote_selection.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1047,6 +1047,114 @@
         <v>466.99</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BOL-40826</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>85</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>C-CRS</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>151.98</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>151.98</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BOL-41318</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="C25" t="n">
+        <v>250</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>C-EXL</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>330.08</v>
+      </c>
+      <c r="F25" t="n">
+        <v>40</v>
+      </c>
+      <c r="G25" t="n">
+        <v>370.08</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BOL-40943</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="C26" t="n">
+        <v>70</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>C-ARW</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>122.38</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>122.38</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BOL-41342</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="C27" t="n">
+        <v>70</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>C-EXL</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>184.74</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>184.74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>